<commit_message>
Auto commit 11-05-2026 12:04:41.50
</commit_message>
<xml_diff>
--- a/Data Base/Global Templates/Well Protection Cover.xlsx
+++ b/Data Base/Global Templates/Well Protection Cover.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manup\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manup\Desktop\estimate-drafter\Data Base\Global Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C58AE1-E85E-4967-89A5-E24806E3991C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F3D6DE-9730-41C4-B487-4A25F0F58DF5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
-  <si>
-    <t>Well Protection Cover</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>Earth work in excavation by mechanical means (Hydraulic excavator)/manual means over areas (exceeding 30 cm in depth, 1.5 m in width as well as 10 sqm on plan) including disposal of excavated earth, lead up to 50 m and lift up to 1.5 m, disposed earth to be levelled and neatly dressed. All kinds of soil (Code: 2.6.1)</t>
   </si>
@@ -110,13 +107,13 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -399,101 +396,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.26953125" style="1" customWidth="1"/>
     <col min="2" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="87" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
-        <v>0.55000000000000004</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="87" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="3">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
-        <v>0.35</v>
+      <c r="B3" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B5" s="4"/>
+    </row>
+    <row r="6" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="B6" s="3">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="B7" s="3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="58" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4">
+      <c r="B8" s="3">
         <v>3.5</v>
       </c>
     </row>
+    <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1.75875</v>
+      </c>
+    </row>
     <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>1.75875</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="4">
-        <v>1.75875</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A6:B6"/>
+  <mergeCells count="1">
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Auto commit 11-05-2026 12:08:37.75
</commit_message>
<xml_diff>
--- a/Data Base/Global Templates/Well Protection Cover.xlsx
+++ b/Data Base/Global Templates/Well Protection Cover.xlsx
@@ -1,31 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manup\Desktop\estimate-drafter\Data Base\Global Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F3D6DE-9730-41C4-B487-4A25F0F58DF5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2A7688-D34C-4914-B4EA-BA5F024895EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+  <si>
+    <t>Well Protection Cover</t>
+  </si>
   <si>
     <t>Earth work in excavation by mechanical means (Hydraulic excavator)/manual means over areas (exceeding 30 cm in depth, 1.5 m in width as well as 10 sqm on plan) including disposal of excavated earth, lead up to 50 m and lift up to 1.5 m, disposed earth to be levelled and neatly dressed. All kinds of soil (Code: 2.6.1)</t>
   </si>
@@ -55,7 +53,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,9 +68,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -77,7 +84,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -87,16 +94,42 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -104,17 +137,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -150,7 +197,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -162,7 +209,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -176,7 +223,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -209,9 +256,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -244,6 +308,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -396,96 +477,103 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.26953125" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="37.81640625" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="4"/>
+    </row>
+    <row r="2" spans="1:2" ht="116" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="87" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3">
+    <row r="3" spans="1:2" ht="101.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7">
         <v>0.35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3">
+    <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+    </row>
+    <row r="5" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+    <row r="6" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:2" ht="101.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="58" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="72.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="7">
+        <v>1.75875</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="43.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4"/>
-    </row>
-    <row r="6" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="3">
+      <c r="B11" s="7">
         <v>1.75875</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="3">
-        <v>1.75875</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A5:B5"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>